<commit_message>
Adicao de historico para planilh
</commit_message>
<xml_diff>
--- a/Financas.xlsx
+++ b/Financas.xlsx
@@ -464,12 +464,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Salario</t>
+          <t>salario</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>29/05/26</t>
+          <t>31/05/26</t>
         </is>
       </c>
     </row>
@@ -487,12 +487,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Aluguel</t>
+          <t>aluguel</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>29/05/26</t>
+          <t>31/05/26</t>
         </is>
       </c>
     </row>
@@ -510,12 +510,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Bico</t>
+          <t>bico</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>29/05/26</t>
+          <t>31/05/26</t>
         </is>
       </c>
     </row>
@@ -533,12 +533,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Banho pet</t>
+          <t>banho pet</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>29/05/26</t>
+          <t>31/05/26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adicao de leitura de extrato de banco
</commit_message>
<xml_diff>
--- a/Financas.xlsx
+++ b/Financas.xlsx
@@ -464,12 +464,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>salario</t>
+          <t>Salario</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>31/05/26</t>
+          <t>29/05/26</t>
         </is>
       </c>
     </row>
@@ -487,12 +487,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>aluguel</t>
+          <t>Aluguel</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>31/05/26</t>
+          <t>29/05/26</t>
         </is>
       </c>
     </row>
@@ -510,12 +510,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>bico</t>
+          <t>Bico</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>31/05/26</t>
+          <t>29/05/26</t>
         </is>
       </c>
     </row>
@@ -533,12 +533,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>banho pet</t>
+          <t>Banho pet</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>31/05/26</t>
+          <t>29/05/26</t>
         </is>
       </c>
     </row>

</xml_diff>